<commit_message>
New Player sprites, weapons & Bug fixes
</commit_message>
<xml_diff>
--- a/docs/balancing.xlsx
+++ b/docs/balancing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5158e6b991fee7f4/Desktop/Schule/Maturarbeit/Godot/matura-roguelite/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="650" documentId="8_{1C25F502-3DF3-4C0E-A964-DFE0638285DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD2B172B-A637-4230-AAC3-DD6D174F7F54}"/>
+  <xr:revisionPtr revIDLastSave="652" documentId="8_{1C25F502-3DF3-4C0E-A964-DFE0638285DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A209D46-F19E-44E5-A108-73993082925F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{5B9A7CE5-9E71-472F-BCC2-975C4625B76B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{5B9A7CE5-9E71-472F-BCC2-975C4625B76B}"/>
   </bookViews>
   <sheets>
     <sheet name="Room Balance" sheetId="1" r:id="rId1"/>

</xml_diff>